<commit_message>
8th commit: Updated BankAccount class with new methods, update_balance, deposit, withdraw and __str__.
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_bank_account.xlsx
+++ b/tests/A01_pixell_test_plan_bank_account.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lauri\Desktop\Intermediate Software Development0315\2. Assignments\updated_again_0416\assignment_01\starter (given)\tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2fbdadfea9c11b5/Documents/rrc-polytech/semester-2/intermediate_software_development/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1849AA10-1E95-48E2-BA5E-F75B35E577F4}"/>
   <bookViews>
-    <workbookView xWindow="31140" yWindow="2340" windowWidth="25185" windowHeight="13845" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="4065" yWindow="1980" windowWidth="21600" windowHeight="12975" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -619,6 +619,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -642,12 +648,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1207,29 +1207,29 @@
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
     </row>
     <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="17"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="19"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="19"/>
+      <c r="D4" s="21"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
@@ -1258,10 +1258,10 @@
       <c r="B7" s="10">
         <v>1</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="11"/>
@@ -1286,10 +1286,10 @@
       <c r="B9" s="13">
         <v>3</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="15" t="s">
         <v>29</v>
       </c>
       <c r="E9" s="12"/>
@@ -1314,10 +1314,10 @@
       <c r="B11" s="10">
         <v>5</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="15" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="12"/>
@@ -1342,10 +1342,10 @@
       <c r="B13" s="3">
         <v>7</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="15" t="s">
         <v>17</v>
       </c>
       <c r="E13" s="12"/>
@@ -1370,10 +1370,10 @@
       <c r="B15" s="10">
         <v>9</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="15" t="s">
         <v>20</v>
       </c>
       <c r="E15" s="12"/>
@@ -1398,10 +1398,10 @@
       <c r="B17" s="10">
         <v>11</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E17" s="12"/>
@@ -1426,10 +1426,10 @@
       <c r="B19" s="13">
         <v>13</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E19" s="12"/>
@@ -1454,10 +1454,10 @@
       <c r="B21" s="10">
         <v>15</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="15" t="s">
         <v>28</v>
       </c>
       <c r="E21" s="4"/>
@@ -1629,14 +1629,14 @@
       <c r="G37" s="5"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
9th commit: Added unittesting for BankAccount class, updated A01_pixell_test_plan_bank_account.xlsx, and updated withdraw and deposit methods in bank_account.py.
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_bank_account.xlsx
+++ b/tests/A01_pixell_test_plan_bank_account.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2fbdadfea9c11b5/Documents/rrc-polytech/semester-2/intermediate_software_development/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1849AA10-1E95-48E2-BA5E-F75B35E577F4}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F3904DF-7C3D-4D99-A86C-9869A2848BBC}"/>
   <bookViews>
-    <workbookView xWindow="4065" yWindow="1980" windowWidth="21600" windowHeight="12975" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="50">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -282,6 +282,65 @@
   </si>
   <si>
     <t>returns client number attribute</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>NOne</t>
+  </si>
+  <si>
+    <t>All attributes are set</t>
+  </si>
+  <si>
+    <t>account_number = 1172007
+client_number = 12345
+balance = 70000.85</t>
+  </si>
+  <si>
+    <t>Balance atrribute set to 0</t>
+  </si>
+  <si>
+    <t>ValueError</t>
+  </si>
+  <si>
+    <t>account_number = 1172007
+client_number = "str"
+balance = 70000.85</t>
+  </si>
+  <si>
+    <t>account_number = "str"
+client_number = 12345
+balance = 70000.85</t>
+  </si>
+  <si>
+    <t>account_number = 1172007
+client_number = 12345
+balance = "str"</t>
+  </si>
+  <si>
+    <t>amount =  500</t>
+  </si>
+  <si>
+    <t>amount =  -500</t>
+  </si>
+  <si>
+    <t>amount = "str"</t>
+  </si>
+  <si>
+    <t>amount = 500</t>
+  </si>
+  <si>
+    <t>amount = -500</t>
+  </si>
+  <si>
+    <t>amount = 80000</t>
+  </si>
+  <si>
+    <t>Account Number: 1172007 Balance: $70,000.85</t>
+  </si>
+  <si>
+    <t>Sven Beitenger</t>
   </si>
 </sst>
 </file>
@@ -588,7 +647,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -649,6 +708,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -794,6 +856,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1219,7 +1285,9 @@
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="18"/>
+      <c r="C3" s="18" t="s">
+        <v>49</v>
+      </c>
       <c r="D3" s="19"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1264,9 +1332,15 @@
       <c r="D7" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
+      <c r="E7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="8" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1278,9 +1352,15 @@
       <c r="D8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="12"/>
+      <c r="E8" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="13">
@@ -1292,9 +1372,15 @@
       <c r="D9" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
+      <c r="E9" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="10">
@@ -1306,9 +1392,15 @@
       <c r="D10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
+      <c r="E10" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="10">
@@ -1320,9 +1412,15 @@
       <c r="D11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
+      <c r="E11" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="12">
+        <v>1172007</v>
+      </c>
     </row>
     <row r="12" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="10">
@@ -1334,9 +1432,15 @@
       <c r="D12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
+      <c r="E12" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="12">
+        <v>12345</v>
+      </c>
     </row>
     <row r="13" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -1348,9 +1452,15 @@
       <c r="D13" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
+      <c r="E13" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="24">
+        <v>70000.850000000006</v>
+      </c>
     </row>
     <row r="14" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="13">
@@ -1362,9 +1472,15 @@
       <c r="D14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
+      <c r="E14" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" s="24">
+        <v>70500.850000000006</v>
+      </c>
     </row>
     <row r="15" spans="2:7" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="10">
@@ -1376,9 +1492,15 @@
       <c r="D15" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="E15" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G15" s="24">
+        <v>69500.850000000006</v>
+      </c>
     </row>
     <row r="16" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="10">
@@ -1390,9 +1512,15 @@
       <c r="D16" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
+      <c r="E16" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G16" s="24">
+        <v>70000.850000000006</v>
+      </c>
     </row>
     <row r="17" spans="2:7" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="10">
@@ -1404,9 +1532,15 @@
       <c r="D17" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
+      <c r="E17" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="24">
+        <v>70500.850000000006</v>
+      </c>
     </row>
     <row r="18" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
@@ -1418,9 +1552,15 @@
       <c r="D18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="E18" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="19" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="13">
@@ -1432,9 +1572,15 @@
       <c r="D19" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
+      <c r="E19" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="24">
+        <v>69500.850000000006</v>
+      </c>
     </row>
     <row r="20" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="10">
@@ -1446,9 +1592,15 @@
       <c r="D20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
+      <c r="E20" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="21" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="10">
@@ -1460,9 +1612,15 @@
       <c r="D21" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="22" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10">
@@ -1474,9 +1632,15 @@
       <c r="D22" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="E22" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="23" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="3">

</xml_diff>